<commit_message>
Added new tests (#1)
* add dev branch

* add back button support

* Add new test
</commit_message>
<xml_diff>
--- a/data/test_data.xlsx
+++ b/data/test_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/leonid/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDE2FB83-4052-C848-8058-2067D36F2CBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C26642E-CED6-7E46-AAA2-0372FB134166}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="27040" windowHeight="15740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="30">
   <si>
     <t>TestID</t>
   </si>
@@ -97,10 +97,19 @@
     <t>TC007</t>
   </si>
   <si>
-    <t>test_library_book_search</t>
-  </si>
-  <si>
     <t>Find the book in library</t>
+  </si>
+  <si>
+    <t>test_library_search_book</t>
+  </si>
+  <si>
+    <t>TC008</t>
+  </si>
+  <si>
+    <t>test_screen_detection</t>
+  </si>
+  <si>
+    <t>Check current screen activity</t>
   </si>
 </sst>
 </file>
@@ -446,7 +455,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6" bestFit="1" customWidth="1"/>
@@ -557,13 +566,27 @@
         <v>24</v>
       </c>
       <c r="B8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C8" t="s">
         <v>6</v>
       </c>
       <c r="D8" t="s">
-        <v>26</v>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>